<commit_message>
Auditoria y seguridad de datos
</commit_message>
<xml_diff>
--- a/Doc_Test/Pruebas_Calidad/Pruebas_Unitarias/CEC-9.xlsx
+++ b/Doc_Test/Pruebas_Calidad/Pruebas_Unitarias/CEC-9.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kevin\Desktop\App_Uv\AppAcompanhamientoUV\Doc_Test\Pruebas_Calidad\Pruebas_Unitarias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8BD7BBB-24CD-457D-992C-233FC203BE43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90F0DEFF-6166-4778-A5B3-C2570170E919}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{2FFDA8E8-6428-4D51-9D6D-F314F8731DBF}"/>
   </bookViews>
@@ -1167,23 +1167,14 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1194,11 +1185,20 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1555,135 +1555,135 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="17"/>
+      <c r="K3" s="17"/>
     </row>
     <row r="4" spans="2:11" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="16">
+      <c r="C5" s="19">
         <v>45849</v>
       </c>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="16"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
     </row>
     <row r="7" spans="2:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="17"/>
     </row>
     <row r="9" spans="2:11" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="18"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="18"/>
     </row>
     <row r="10" spans="2:11" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="14"/>
+      <c r="C10" s="21"/>
       <c r="D10" s="6" t="s">
         <v>6</v>
       </c>
@@ -1710,23 +1710,23 @@
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="15"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13"/>
+      <c r="K11" s="13"/>
     </row>
     <row r="12" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B12" s="17"/>
+      <c r="B12" s="14"/>
       <c r="C12" s="7" t="s">
         <v>15</v>
       </c>
@@ -1745,16 +1745,16 @@
       <c r="H12" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I12" s="19" t="s">
+      <c r="I12" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="J12" s="19" t="s">
+      <c r="J12" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K12" s="18"/>
+      <c r="K12" s="15"/>
     </row>
     <row r="13" spans="2:11" ht="199.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="17"/>
+      <c r="B13" s="14"/>
       <c r="C13" s="9" t="s">
         <v>16</v>
       </c>
@@ -1773,12 +1773,12 @@
       <c r="H13" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I13" s="19"/>
-      <c r="J13" s="19"/>
-      <c r="K13" s="18"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="15"/>
     </row>
     <row r="14" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B14" s="17"/>
+      <c r="B14" s="14"/>
       <c r="C14" s="9" t="s">
         <v>19</v>
       </c>
@@ -1797,12 +1797,12 @@
       <c r="H14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I14" s="19"/>
-      <c r="J14" s="19"/>
-      <c r="K14" s="18"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="15"/>
     </row>
     <row r="15" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B15" s="17"/>
+      <c r="B15" s="14"/>
       <c r="C15" s="9" t="s">
         <v>35</v>
       </c>
@@ -1821,12 +1821,12 @@
       <c r="H15" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I15" s="19"/>
-      <c r="J15" s="19"/>
-      <c r="K15" s="18"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="15"/>
     </row>
     <row r="16" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B16" s="17"/>
+      <c r="B16" s="14"/>
       <c r="C16" s="9" t="s">
         <v>36</v>
       </c>
@@ -1845,12 +1845,12 @@
       <c r="H16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I16" s="19"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="18"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="15"/>
     </row>
     <row r="17" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B17" s="17"/>
+      <c r="B17" s="14"/>
       <c r="C17" s="9" t="s">
         <v>37</v>
       </c>
@@ -1869,12 +1869,12 @@
       <c r="H17" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I17" s="19"/>
-      <c r="J17" s="19"/>
-      <c r="K17" s="18"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="15"/>
     </row>
     <row r="18" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B18" s="17"/>
+      <c r="B18" s="14"/>
       <c r="C18" s="9" t="s">
         <v>37</v>
       </c>
@@ -1893,28 +1893,28 @@
       <c r="H18" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I18" s="19"/>
-      <c r="J18" s="19"/>
-      <c r="K18" s="18"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="15"/>
     </row>
     <row r="19" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="15"/>
-      <c r="J19" s="15"/>
-      <c r="K19" s="15"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13"/>
     </row>
     <row r="20" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B20" s="17"/>
+      <c r="B20" s="14"/>
       <c r="C20" s="7" t="s">
         <v>25</v>
       </c>
@@ -1933,16 +1933,16 @@
       <c r="H20" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I20" s="19" t="s">
+      <c r="I20" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="J20" s="19" t="s">
+      <c r="J20" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K20" s="18"/>
+      <c r="K20" s="15"/>
     </row>
     <row r="21" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B21" s="17"/>
+      <c r="B21" s="14"/>
       <c r="C21" s="7" t="s">
         <v>26</v>
       </c>
@@ -1961,12 +1961,12 @@
       <c r="H21" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I21" s="19"/>
-      <c r="J21" s="19"/>
-      <c r="K21" s="18"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="15"/>
     </row>
     <row r="22" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B22" s="17"/>
+      <c r="B22" s="14"/>
       <c r="C22" s="7" t="s">
         <v>27</v>
       </c>
@@ -1985,12 +1985,12 @@
       <c r="H22" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I22" s="19"/>
-      <c r="J22" s="19"/>
-      <c r="K22" s="18"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="15"/>
     </row>
     <row r="23" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B23" s="17"/>
+      <c r="B23" s="14"/>
       <c r="C23" s="7" t="s">
         <v>55</v>
       </c>
@@ -2009,12 +2009,12 @@
       <c r="H23" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
-      <c r="K23" s="18"/>
+      <c r="I23" s="16"/>
+      <c r="J23" s="16"/>
+      <c r="K23" s="15"/>
     </row>
     <row r="24" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B24" s="17"/>
+      <c r="B24" s="14"/>
       <c r="C24" s="7" t="s">
         <v>56</v>
       </c>
@@ -2033,12 +2033,12 @@
       <c r="H24" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I24" s="19"/>
-      <c r="J24" s="19"/>
-      <c r="K24" s="18"/>
+      <c r="I24" s="16"/>
+      <c r="J24" s="16"/>
+      <c r="K24" s="15"/>
     </row>
     <row r="25" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B25" s="17"/>
+      <c r="B25" s="14"/>
       <c r="C25" s="7" t="s">
         <v>60</v>
       </c>
@@ -2057,28 +2057,28 @@
       <c r="H25" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I25" s="19"/>
-      <c r="J25" s="19"/>
-      <c r="K25" s="18"/>
+      <c r="I25" s="16"/>
+      <c r="J25" s="16"/>
+      <c r="K25" s="15"/>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="C26" s="15" t="s">
+      <c r="C26" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="15"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="15"/>
-      <c r="J26" s="15"/>
-      <c r="K26" s="15"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
     </row>
     <row r="27" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B27" s="17"/>
+      <c r="B27" s="14"/>
       <c r="C27" s="7" t="s">
         <v>63</v>
       </c>
@@ -2097,18 +2097,18 @@
       <c r="H27" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I27" s="18" t="s">
+      <c r="I27" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="J27" s="19" t="s">
+      <c r="J27" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K27" s="18" t="s">
+      <c r="K27" s="15" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="28" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B28" s="17"/>
+      <c r="B28" s="14"/>
       <c r="C28" s="7" t="s">
         <v>64</v>
       </c>
@@ -2127,12 +2127,12 @@
       <c r="H28" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I28" s="18"/>
-      <c r="J28" s="19"/>
-      <c r="K28" s="18"/>
+      <c r="I28" s="15"/>
+      <c r="J28" s="16"/>
+      <c r="K28" s="15"/>
     </row>
     <row r="29" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B29" s="17"/>
+      <c r="B29" s="14"/>
       <c r="C29" s="7" t="s">
         <v>65</v>
       </c>
@@ -2151,12 +2151,12 @@
       <c r="H29" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I29" s="18"/>
-      <c r="J29" s="19"/>
-      <c r="K29" s="18"/>
+      <c r="I29" s="15"/>
+      <c r="J29" s="16"/>
+      <c r="K29" s="15"/>
     </row>
     <row r="30" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B30" s="17"/>
+      <c r="B30" s="14"/>
       <c r="C30" s="7" t="s">
         <v>66</v>
       </c>
@@ -2175,12 +2175,12 @@
       <c r="H30" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I30" s="18"/>
-      <c r="J30" s="19"/>
-      <c r="K30" s="18"/>
+      <c r="I30" s="15"/>
+      <c r="J30" s="16"/>
+      <c r="K30" s="15"/>
     </row>
     <row r="31" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B31" s="17"/>
+      <c r="B31" s="14"/>
       <c r="C31" s="7" t="s">
         <v>67</v>
       </c>
@@ -2199,12 +2199,12 @@
       <c r="H31" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I31" s="18"/>
-      <c r="J31" s="19"/>
-      <c r="K31" s="18"/>
+      <c r="I31" s="15"/>
+      <c r="J31" s="16"/>
+      <c r="K31" s="15"/>
     </row>
     <row r="32" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B32" s="17"/>
+      <c r="B32" s="14"/>
       <c r="C32" s="7" t="s">
         <v>68</v>
       </c>
@@ -2223,12 +2223,12 @@
       <c r="H32" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I32" s="18"/>
-      <c r="J32" s="19"/>
-      <c r="K32" s="18"/>
+      <c r="I32" s="15"/>
+      <c r="J32" s="16"/>
+      <c r="K32" s="15"/>
     </row>
     <row r="33" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B33" s="17"/>
+      <c r="B33" s="14"/>
       <c r="C33" s="7" t="s">
         <v>69</v>
       </c>
@@ -2247,28 +2247,28 @@
       <c r="H33" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I33" s="18"/>
-      <c r="J33" s="19"/>
-      <c r="K33" s="18"/>
+      <c r="I33" s="15"/>
+      <c r="J33" s="16"/>
+      <c r="K33" s="15"/>
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B34" s="17" t="s">
+      <c r="B34" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="C34" s="15" t="s">
+      <c r="C34" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="D34" s="15"/>
-      <c r="E34" s="15"/>
-      <c r="F34" s="15"/>
-      <c r="G34" s="15"/>
-      <c r="H34" s="15"/>
-      <c r="I34" s="15"/>
-      <c r="J34" s="15"/>
-      <c r="K34" s="15"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="13"/>
+      <c r="F34" s="13"/>
+      <c r="G34" s="13"/>
+      <c r="H34" s="13"/>
+      <c r="I34" s="13"/>
+      <c r="J34" s="13"/>
+      <c r="K34" s="13"/>
     </row>
     <row r="35" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B35" s="17"/>
+      <c r="B35" s="14"/>
       <c r="C35" s="7" t="s">
         <v>72</v>
       </c>
@@ -2287,18 +2287,18 @@
       <c r="H35" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I35" s="18" t="s">
+      <c r="I35" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="J35" s="19" t="s">
+      <c r="J35" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K35" s="18" t="s">
+      <c r="K35" s="15" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="36" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B36" s="17"/>
+      <c r="B36" s="14"/>
       <c r="C36" s="7" t="s">
         <v>73</v>
       </c>
@@ -2317,12 +2317,12 @@
       <c r="H36" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I36" s="18"/>
-      <c r="J36" s="19"/>
-      <c r="K36" s="18"/>
+      <c r="I36" s="15"/>
+      <c r="J36" s="16"/>
+      <c r="K36" s="15"/>
     </row>
     <row r="37" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B37" s="17"/>
+      <c r="B37" s="14"/>
       <c r="C37" s="7" t="s">
         <v>74</v>
       </c>
@@ -2341,12 +2341,12 @@
       <c r="H37" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I37" s="18"/>
-      <c r="J37" s="19"/>
-      <c r="K37" s="18"/>
+      <c r="I37" s="15"/>
+      <c r="J37" s="16"/>
+      <c r="K37" s="15"/>
     </row>
     <row r="38" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B38" s="17"/>
+      <c r="B38" s="14"/>
       <c r="C38" s="7" t="s">
         <v>75</v>
       </c>
@@ -2365,12 +2365,12 @@
       <c r="H38" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I38" s="18"/>
-      <c r="J38" s="19"/>
-      <c r="K38" s="18"/>
+      <c r="I38" s="15"/>
+      <c r="J38" s="16"/>
+      <c r="K38" s="15"/>
     </row>
     <row r="39" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B39" s="17"/>
+      <c r="B39" s="14"/>
       <c r="C39" s="7" t="s">
         <v>76</v>
       </c>
@@ -2389,12 +2389,12 @@
       <c r="H39" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I39" s="18"/>
-      <c r="J39" s="19"/>
-      <c r="K39" s="18"/>
+      <c r="I39" s="15"/>
+      <c r="J39" s="16"/>
+      <c r="K39" s="15"/>
     </row>
     <row r="40" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B40" s="17"/>
+      <c r="B40" s="14"/>
       <c r="C40" s="7" t="s">
         <v>77</v>
       </c>
@@ -2413,28 +2413,28 @@
       <c r="H40" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I40" s="18"/>
-      <c r="J40" s="19"/>
-      <c r="K40" s="18"/>
+      <c r="I40" s="15"/>
+      <c r="J40" s="16"/>
+      <c r="K40" s="15"/>
     </row>
     <row r="41" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B41" s="17" t="s">
+      <c r="B41" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="15" t="s">
+      <c r="C41" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="D41" s="15"/>
-      <c r="E41" s="15"/>
-      <c r="F41" s="15"/>
-      <c r="G41" s="15"/>
-      <c r="H41" s="15"/>
-      <c r="I41" s="15"/>
-      <c r="J41" s="15"/>
-      <c r="K41" s="15"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="13"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
+      <c r="H41" s="13"/>
+      <c r="I41" s="13"/>
+      <c r="J41" s="13"/>
+      <c r="K41" s="13"/>
     </row>
     <row r="42" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B42" s="17"/>
+      <c r="B42" s="14"/>
       <c r="C42" s="7" t="s">
         <v>83</v>
       </c>
@@ -2453,16 +2453,16 @@
       <c r="H42" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I42" s="19" t="s">
+      <c r="I42" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="J42" s="19" t="s">
+      <c r="J42" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K42" s="18"/>
+      <c r="K42" s="15"/>
     </row>
     <row r="43" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B43" s="17"/>
+      <c r="B43" s="14"/>
       <c r="C43" s="7" t="s">
         <v>84</v>
       </c>
@@ -2481,12 +2481,12 @@
       <c r="H43" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I43" s="19"/>
-      <c r="J43" s="19"/>
-      <c r="K43" s="18"/>
+      <c r="I43" s="16"/>
+      <c r="J43" s="16"/>
+      <c r="K43" s="15"/>
     </row>
     <row r="44" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B44" s="17"/>
+      <c r="B44" s="14"/>
       <c r="C44" s="7" t="s">
         <v>85</v>
       </c>
@@ -2505,12 +2505,12 @@
       <c r="H44" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I44" s="19"/>
-      <c r="J44" s="19"/>
-      <c r="K44" s="18"/>
+      <c r="I44" s="16"/>
+      <c r="J44" s="16"/>
+      <c r="K44" s="15"/>
     </row>
     <row r="45" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B45" s="17"/>
+      <c r="B45" s="14"/>
       <c r="C45" s="7" t="s">
         <v>86</v>
       </c>
@@ -2529,12 +2529,12 @@
       <c r="H45" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I45" s="19"/>
-      <c r="J45" s="19"/>
-      <c r="K45" s="18"/>
+      <c r="I45" s="16"/>
+      <c r="J45" s="16"/>
+      <c r="K45" s="15"/>
     </row>
     <row r="46" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B46" s="17"/>
+      <c r="B46" s="14"/>
       <c r="C46" s="7" t="s">
         <v>87</v>
       </c>
@@ -2553,12 +2553,12 @@
       <c r="H46" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I46" s="19"/>
-      <c r="J46" s="19"/>
-      <c r="K46" s="18"/>
+      <c r="I46" s="16"/>
+      <c r="J46" s="16"/>
+      <c r="K46" s="15"/>
     </row>
     <row r="47" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B47" s="17"/>
+      <c r="B47" s="14"/>
       <c r="C47" s="7" t="s">
         <v>88</v>
       </c>
@@ -2577,28 +2577,28 @@
       <c r="H47" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I47" s="19"/>
-      <c r="J47" s="19"/>
-      <c r="K47" s="18"/>
+      <c r="I47" s="16"/>
+      <c r="J47" s="16"/>
+      <c r="K47" s="15"/>
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B48" s="17" t="s">
+      <c r="B48" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="C48" s="15" t="s">
+      <c r="C48" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="D48" s="15"/>
-      <c r="E48" s="15"/>
-      <c r="F48" s="15"/>
-      <c r="G48" s="15"/>
-      <c r="H48" s="15"/>
-      <c r="I48" s="15"/>
-      <c r="J48" s="15"/>
-      <c r="K48" s="15"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="13"/>
+      <c r="F48" s="13"/>
+      <c r="G48" s="13"/>
+      <c r="H48" s="13"/>
+      <c r="I48" s="13"/>
+      <c r="J48" s="13"/>
+      <c r="K48" s="13"/>
     </row>
     <row r="49" spans="2:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="17"/>
+      <c r="B49" s="14"/>
       <c r="C49" s="7" t="s">
         <v>72</v>
       </c>
@@ -2617,16 +2617,16 @@
       <c r="H49" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I49" s="19" t="s">
+      <c r="I49" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="J49" s="19" t="s">
+      <c r="J49" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K49" s="18"/>
+      <c r="K49" s="15"/>
     </row>
     <row r="50" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B50" s="17"/>
+      <c r="B50" s="14"/>
       <c r="C50" s="7" t="s">
         <v>73</v>
       </c>
@@ -2645,12 +2645,12 @@
       <c r="H50" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I50" s="19"/>
-      <c r="J50" s="19"/>
-      <c r="K50" s="18"/>
+      <c r="I50" s="16"/>
+      <c r="J50" s="16"/>
+      <c r="K50" s="15"/>
     </row>
     <row r="51" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B51" s="17"/>
+      <c r="B51" s="14"/>
       <c r="C51" s="7" t="s">
         <v>74</v>
       </c>
@@ -2669,12 +2669,12 @@
       <c r="H51" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I51" s="19"/>
-      <c r="J51" s="19"/>
-      <c r="K51" s="18"/>
+      <c r="I51" s="16"/>
+      <c r="J51" s="16"/>
+      <c r="K51" s="15"/>
     </row>
     <row r="52" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B52" s="17"/>
+      <c r="B52" s="14"/>
       <c r="C52" s="7" t="s">
         <v>75</v>
       </c>
@@ -2693,12 +2693,12 @@
       <c r="H52" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I52" s="19"/>
-      <c r="J52" s="19"/>
-      <c r="K52" s="18"/>
+      <c r="I52" s="16"/>
+      <c r="J52" s="16"/>
+      <c r="K52" s="15"/>
     </row>
     <row r="53" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B53" s="17"/>
+      <c r="B53" s="14"/>
       <c r="C53" s="7" t="s">
         <v>77</v>
       </c>
@@ -2717,28 +2717,28 @@
       <c r="H53" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I53" s="19"/>
-      <c r="J53" s="19"/>
-      <c r="K53" s="18"/>
+      <c r="I53" s="16"/>
+      <c r="J53" s="16"/>
+      <c r="K53" s="15"/>
     </row>
     <row r="54" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B54" s="17" t="s">
+      <c r="B54" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="C54" s="15" t="s">
+      <c r="C54" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="D54" s="15"/>
-      <c r="E54" s="15"/>
-      <c r="F54" s="15"/>
-      <c r="G54" s="15"/>
-      <c r="H54" s="15"/>
-      <c r="I54" s="15"/>
-      <c r="J54" s="15"/>
-      <c r="K54" s="15"/>
+      <c r="D54" s="13"/>
+      <c r="E54" s="13"/>
+      <c r="F54" s="13"/>
+      <c r="G54" s="13"/>
+      <c r="H54" s="13"/>
+      <c r="I54" s="13"/>
+      <c r="J54" s="13"/>
+      <c r="K54" s="13"/>
     </row>
     <row r="55" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B55" s="17"/>
+      <c r="B55" s="14"/>
       <c r="C55" s="7" t="s">
         <v>83</v>
       </c>
@@ -2757,18 +2757,18 @@
       <c r="H55" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I55" s="18" t="s">
+      <c r="I55" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="J55" s="19" t="s">
+      <c r="J55" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K55" s="18" t="s">
+      <c r="K55" s="15" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="56" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B56" s="17"/>
+      <c r="B56" s="14"/>
       <c r="C56" s="7" t="s">
         <v>84</v>
       </c>
@@ -2787,12 +2787,12 @@
       <c r="H56" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I56" s="18"/>
-      <c r="J56" s="19"/>
-      <c r="K56" s="18"/>
+      <c r="I56" s="15"/>
+      <c r="J56" s="16"/>
+      <c r="K56" s="15"/>
     </row>
     <row r="57" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B57" s="17"/>
+      <c r="B57" s="14"/>
       <c r="C57" s="7" t="s">
         <v>85</v>
       </c>
@@ -2811,12 +2811,12 @@
       <c r="H57" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I57" s="18"/>
-      <c r="J57" s="19"/>
-      <c r="K57" s="18"/>
+      <c r="I57" s="15"/>
+      <c r="J57" s="16"/>
+      <c r="K57" s="15"/>
     </row>
     <row r="58" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B58" s="17"/>
+      <c r="B58" s="14"/>
       <c r="C58" s="7" t="s">
         <v>86</v>
       </c>
@@ -2835,12 +2835,12 @@
       <c r="H58" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I58" s="18"/>
-      <c r="J58" s="19"/>
-      <c r="K58" s="18"/>
+      <c r="I58" s="15"/>
+      <c r="J58" s="16"/>
+      <c r="K58" s="15"/>
     </row>
     <row r="59" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B59" s="17"/>
+      <c r="B59" s="14"/>
       <c r="C59" s="7" t="s">
         <v>87</v>
       </c>
@@ -2859,12 +2859,12 @@
       <c r="H59" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I59" s="18"/>
-      <c r="J59" s="19"/>
-      <c r="K59" s="18"/>
+      <c r="I59" s="15"/>
+      <c r="J59" s="16"/>
+      <c r="K59" s="15"/>
     </row>
     <row r="60" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B60" s="17"/>
+      <c r="B60" s="14"/>
       <c r="C60" s="7" t="s">
         <v>88</v>
       </c>
@@ -2883,28 +2883,28 @@
       <c r="H60" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I60" s="18"/>
-      <c r="J60" s="19"/>
-      <c r="K60" s="18"/>
+      <c r="I60" s="15"/>
+      <c r="J60" s="16"/>
+      <c r="K60" s="15"/>
     </row>
     <row r="61" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B61" s="17" t="s">
+      <c r="B61" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="C61" s="15" t="s">
+      <c r="C61" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="D61" s="15"/>
-      <c r="E61" s="15"/>
-      <c r="F61" s="15"/>
-      <c r="G61" s="15"/>
-      <c r="H61" s="15"/>
-      <c r="I61" s="15"/>
-      <c r="J61" s="15"/>
-      <c r="K61" s="15"/>
+      <c r="D61" s="13"/>
+      <c r="E61" s="13"/>
+      <c r="F61" s="13"/>
+      <c r="G61" s="13"/>
+      <c r="H61" s="13"/>
+      <c r="I61" s="13"/>
+      <c r="J61" s="13"/>
+      <c r="K61" s="13"/>
     </row>
     <row r="62" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B62" s="17"/>
+      <c r="B62" s="14"/>
       <c r="C62" s="7" t="s">
         <v>91</v>
       </c>
@@ -2923,18 +2923,18 @@
       <c r="H62" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I62" s="18" t="s">
+      <c r="I62" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="J62" s="19" t="s">
+      <c r="J62" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K62" s="18" t="s">
+      <c r="K62" s="15" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="63" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B63" s="17"/>
+      <c r="B63" s="14"/>
       <c r="C63" s="7" t="s">
         <v>92</v>
       </c>
@@ -2953,12 +2953,12 @@
       <c r="H63" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I63" s="18"/>
-      <c r="J63" s="19"/>
-      <c r="K63" s="18"/>
+      <c r="I63" s="15"/>
+      <c r="J63" s="16"/>
+      <c r="K63" s="15"/>
     </row>
     <row r="64" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B64" s="17"/>
+      <c r="B64" s="14"/>
       <c r="C64" s="7" t="s">
         <v>93</v>
       </c>
@@ -2977,12 +2977,12 @@
       <c r="H64" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I64" s="18"/>
-      <c r="J64" s="19"/>
-      <c r="K64" s="18"/>
+      <c r="I64" s="15"/>
+      <c r="J64" s="16"/>
+      <c r="K64" s="15"/>
     </row>
     <row r="65" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B65" s="17"/>
+      <c r="B65" s="14"/>
       <c r="C65" s="7" t="s">
         <v>94</v>
       </c>
@@ -3001,12 +3001,12 @@
       <c r="H65" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I65" s="18"/>
-      <c r="J65" s="19"/>
-      <c r="K65" s="18"/>
+      <c r="I65" s="15"/>
+      <c r="J65" s="16"/>
+      <c r="K65" s="15"/>
     </row>
     <row r="66" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B66" s="17"/>
+      <c r="B66" s="14"/>
       <c r="C66" s="7" t="s">
         <v>95</v>
       </c>
@@ -3025,28 +3025,28 @@
       <c r="H66" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I66" s="18"/>
-      <c r="J66" s="19"/>
-      <c r="K66" s="18"/>
+      <c r="I66" s="15"/>
+      <c r="J66" s="16"/>
+      <c r="K66" s="15"/>
     </row>
     <row r="67" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B67" s="17" t="s">
+      <c r="B67" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="C67" s="15" t="s">
+      <c r="C67" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="D67" s="15"/>
-      <c r="E67" s="15"/>
-      <c r="F67" s="15"/>
-      <c r="G67" s="15"/>
-      <c r="H67" s="15"/>
-      <c r="I67" s="15"/>
-      <c r="J67" s="15"/>
-      <c r="K67" s="15"/>
+      <c r="D67" s="13"/>
+      <c r="E67" s="13"/>
+      <c r="F67" s="13"/>
+      <c r="G67" s="13"/>
+      <c r="H67" s="13"/>
+      <c r="I67" s="13"/>
+      <c r="J67" s="13"/>
+      <c r="K67" s="13"/>
     </row>
     <row r="68" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B68" s="17"/>
+      <c r="B68" s="14"/>
       <c r="C68" s="7" t="s">
         <v>100</v>
       </c>
@@ -3065,16 +3065,16 @@
       <c r="H68" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I68" s="19" t="s">
+      <c r="I68" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="J68" s="19" t="s">
+      <c r="J68" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K68" s="18"/>
+      <c r="K68" s="15"/>
     </row>
     <row r="69" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B69" s="17"/>
+      <c r="B69" s="14"/>
       <c r="C69" s="7" t="s">
         <v>101</v>
       </c>
@@ -3093,12 +3093,12 @@
       <c r="H69" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I69" s="19"/>
-      <c r="J69" s="19"/>
-      <c r="K69" s="18"/>
+      <c r="I69" s="16"/>
+      <c r="J69" s="16"/>
+      <c r="K69" s="15"/>
     </row>
     <row r="70" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B70" s="17"/>
+      <c r="B70" s="14"/>
       <c r="C70" s="7" t="s">
         <v>102</v>
       </c>
@@ -3117,12 +3117,12 @@
       <c r="H70" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I70" s="19"/>
-      <c r="J70" s="19"/>
-      <c r="K70" s="18"/>
+      <c r="I70" s="16"/>
+      <c r="J70" s="16"/>
+      <c r="K70" s="15"/>
     </row>
     <row r="71" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B71" s="17"/>
+      <c r="B71" s="14"/>
       <c r="C71" s="7" t="s">
         <v>103</v>
       </c>
@@ -3141,12 +3141,12 @@
       <c r="H71" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I71" s="19"/>
-      <c r="J71" s="19"/>
-      <c r="K71" s="18"/>
+      <c r="I71" s="16"/>
+      <c r="J71" s="16"/>
+      <c r="K71" s="15"/>
     </row>
     <row r="72" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B72" s="17"/>
+      <c r="B72" s="14"/>
       <c r="C72" s="7" t="s">
         <v>104</v>
       </c>
@@ -3165,28 +3165,28 @@
       <c r="H72" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I72" s="19"/>
-      <c r="J72" s="19"/>
-      <c r="K72" s="18"/>
+      <c r="I72" s="16"/>
+      <c r="J72" s="16"/>
+      <c r="K72" s="15"/>
     </row>
     <row r="73" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B73" s="17" t="s">
+      <c r="B73" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="C73" s="15" t="s">
+      <c r="C73" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="D73" s="15"/>
-      <c r="E73" s="15"/>
-      <c r="F73" s="15"/>
-      <c r="G73" s="15"/>
-      <c r="H73" s="15"/>
-      <c r="I73" s="15"/>
-      <c r="J73" s="15"/>
-      <c r="K73" s="15"/>
+      <c r="D73" s="13"/>
+      <c r="E73" s="13"/>
+      <c r="F73" s="13"/>
+      <c r="G73" s="13"/>
+      <c r="H73" s="13"/>
+      <c r="I73" s="13"/>
+      <c r="J73" s="13"/>
+      <c r="K73" s="13"/>
     </row>
     <row r="74" spans="2:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B74" s="17"/>
+      <c r="B74" s="14"/>
       <c r="C74" s="7" t="s">
         <v>117</v>
       </c>
@@ -3205,18 +3205,18 @@
       <c r="H74" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I74" s="18" t="s">
+      <c r="I74" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="J74" s="19" t="s">
+      <c r="J74" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K74" s="18" t="s">
+      <c r="K74" s="15" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="75" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B75" s="17"/>
+      <c r="B75" s="14"/>
       <c r="C75" s="7" t="s">
         <v>118</v>
       </c>
@@ -3235,12 +3235,12 @@
       <c r="H75" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I75" s="18"/>
-      <c r="J75" s="19"/>
-      <c r="K75" s="18"/>
+      <c r="I75" s="15"/>
+      <c r="J75" s="16"/>
+      <c r="K75" s="15"/>
     </row>
     <row r="76" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B76" s="17"/>
+      <c r="B76" s="14"/>
       <c r="C76" s="7" t="s">
         <v>119</v>
       </c>
@@ -3259,12 +3259,12 @@
       <c r="H76" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I76" s="18"/>
-      <c r="J76" s="19"/>
-      <c r="K76" s="18"/>
+      <c r="I76" s="15"/>
+      <c r="J76" s="16"/>
+      <c r="K76" s="15"/>
     </row>
     <row r="77" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B77" s="17"/>
+      <c r="B77" s="14"/>
       <c r="C77" s="7" t="s">
         <v>120</v>
       </c>
@@ -3283,12 +3283,12 @@
       <c r="H77" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I77" s="18"/>
-      <c r="J77" s="19"/>
-      <c r="K77" s="18"/>
+      <c r="I77" s="15"/>
+      <c r="J77" s="16"/>
+      <c r="K77" s="15"/>
     </row>
     <row r="78" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B78" s="17"/>
+      <c r="B78" s="14"/>
       <c r="C78" s="7" t="s">
         <v>121</v>
       </c>
@@ -3307,12 +3307,12 @@
       <c r="H78" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I78" s="18"/>
-      <c r="J78" s="19"/>
-      <c r="K78" s="18"/>
+      <c r="I78" s="15"/>
+      <c r="J78" s="16"/>
+      <c r="K78" s="15"/>
     </row>
     <row r="79" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B79" s="17"/>
+      <c r="B79" s="14"/>
       <c r="C79" s="7" t="s">
         <v>122</v>
       </c>
@@ -3331,12 +3331,12 @@
       <c r="H79" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I79" s="18"/>
-      <c r="J79" s="19"/>
-      <c r="K79" s="18"/>
+      <c r="I79" s="15"/>
+      <c r="J79" s="16"/>
+      <c r="K79" s="15"/>
     </row>
     <row r="80" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B80" s="17"/>
+      <c r="B80" s="14"/>
       <c r="C80" s="7" t="s">
         <v>123</v>
       </c>
@@ -3355,12 +3355,12 @@
       <c r="H80" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I80" s="18"/>
-      <c r="J80" s="19"/>
-      <c r="K80" s="18"/>
+      <c r="I80" s="15"/>
+      <c r="J80" s="16"/>
+      <c r="K80" s="15"/>
     </row>
     <row r="81" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B81" s="17"/>
+      <c r="B81" s="14"/>
       <c r="C81" s="7" t="s">
         <v>124</v>
       </c>
@@ -3379,28 +3379,28 @@
       <c r="H81" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I81" s="18"/>
-      <c r="J81" s="19"/>
-      <c r="K81" s="18"/>
+      <c r="I81" s="15"/>
+      <c r="J81" s="16"/>
+      <c r="K81" s="15"/>
     </row>
     <row r="82" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B82" s="17" t="s">
+      <c r="B82" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="C82" s="15" t="s">
+      <c r="C82" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="D82" s="15"/>
-      <c r="E82" s="15"/>
-      <c r="F82" s="15"/>
-      <c r="G82" s="15"/>
-      <c r="H82" s="15"/>
-      <c r="I82" s="15"/>
-      <c r="J82" s="15"/>
-      <c r="K82" s="15"/>
+      <c r="D82" s="13"/>
+      <c r="E82" s="13"/>
+      <c r="F82" s="13"/>
+      <c r="G82" s="13"/>
+      <c r="H82" s="13"/>
+      <c r="I82" s="13"/>
+      <c r="J82" s="13"/>
+      <c r="K82" s="13"/>
     </row>
     <row r="83" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B83" s="17"/>
+      <c r="B83" s="14"/>
       <c r="C83" s="7" t="s">
         <v>131</v>
       </c>
@@ -3419,18 +3419,18 @@
       <c r="H83" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I83" s="18" t="s">
+      <c r="I83" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="J83" s="19" t="s">
+      <c r="J83" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K83" s="18" t="s">
+      <c r="K83" s="15" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="84" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B84" s="17"/>
+      <c r="B84" s="14"/>
       <c r="C84" s="7" t="s">
         <v>132</v>
       </c>
@@ -3449,12 +3449,12 @@
       <c r="H84" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I84" s="18"/>
-      <c r="J84" s="19"/>
-      <c r="K84" s="18"/>
+      <c r="I84" s="15"/>
+      <c r="J84" s="16"/>
+      <c r="K84" s="15"/>
     </row>
     <row r="85" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B85" s="17"/>
+      <c r="B85" s="14"/>
       <c r="C85" s="7" t="s">
         <v>133</v>
       </c>
@@ -3473,12 +3473,12 @@
       <c r="H85" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I85" s="18"/>
-      <c r="J85" s="19"/>
-      <c r="K85" s="18"/>
+      <c r="I85" s="15"/>
+      <c r="J85" s="16"/>
+      <c r="K85" s="15"/>
     </row>
     <row r="86" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B86" s="17"/>
+      <c r="B86" s="14"/>
       <c r="C86" s="7" t="s">
         <v>134</v>
       </c>
@@ -3497,12 +3497,12 @@
       <c r="H86" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I86" s="18"/>
-      <c r="J86" s="19"/>
-      <c r="K86" s="18"/>
+      <c r="I86" s="15"/>
+      <c r="J86" s="16"/>
+      <c r="K86" s="15"/>
     </row>
     <row r="87" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B87" s="17"/>
+      <c r="B87" s="14"/>
       <c r="C87" s="7" t="s">
         <v>135</v>
       </c>
@@ -3521,12 +3521,12 @@
       <c r="H87" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I87" s="18"/>
-      <c r="J87" s="19"/>
-      <c r="K87" s="18"/>
+      <c r="I87" s="15"/>
+      <c r="J87" s="16"/>
+      <c r="K87" s="15"/>
     </row>
     <row r="88" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B88" s="17"/>
+      <c r="B88" s="14"/>
       <c r="C88" s="7" t="s">
         <v>136</v>
       </c>
@@ -3545,12 +3545,12 @@
       <c r="H88" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I88" s="18"/>
-      <c r="J88" s="19"/>
-      <c r="K88" s="18"/>
+      <c r="I88" s="15"/>
+      <c r="J88" s="16"/>
+      <c r="K88" s="15"/>
     </row>
     <row r="89" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B89" s="17"/>
+      <c r="B89" s="14"/>
       <c r="C89" s="7" t="s">
         <v>137</v>
       </c>
@@ -3569,28 +3569,28 @@
       <c r="H89" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I89" s="18"/>
-      <c r="J89" s="19"/>
-      <c r="K89" s="18"/>
+      <c r="I89" s="15"/>
+      <c r="J89" s="16"/>
+      <c r="K89" s="15"/>
     </row>
     <row r="90" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B90" s="17" t="s">
+      <c r="B90" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="C90" s="15" t="s">
+      <c r="C90" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="D90" s="15"/>
-      <c r="E90" s="15"/>
-      <c r="F90" s="15"/>
-      <c r="G90" s="15"/>
-      <c r="H90" s="15"/>
-      <c r="I90" s="15"/>
-      <c r="J90" s="15"/>
-      <c r="K90" s="15"/>
+      <c r="D90" s="13"/>
+      <c r="E90" s="13"/>
+      <c r="F90" s="13"/>
+      <c r="G90" s="13"/>
+      <c r="H90" s="13"/>
+      <c r="I90" s="13"/>
+      <c r="J90" s="13"/>
+      <c r="K90" s="13"/>
     </row>
     <row r="91" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B91" s="17"/>
+      <c r="B91" s="14"/>
       <c r="C91" s="7" t="s">
         <v>143</v>
       </c>
@@ -3609,16 +3609,16 @@
       <c r="H91" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I91" s="18" t="s">
+      <c r="I91" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="J91" s="19" t="s">
+      <c r="J91" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K91" s="18"/>
+      <c r="K91" s="15"/>
     </row>
     <row r="92" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B92" s="17"/>
+      <c r="B92" s="14"/>
       <c r="C92" s="7" t="s">
         <v>144</v>
       </c>
@@ -3637,12 +3637,12 @@
       <c r="H92" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I92" s="18"/>
-      <c r="J92" s="19"/>
-      <c r="K92" s="18"/>
+      <c r="I92" s="15"/>
+      <c r="J92" s="16"/>
+      <c r="K92" s="15"/>
     </row>
     <row r="93" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B93" s="17"/>
+      <c r="B93" s="14"/>
       <c r="C93" s="7" t="s">
         <v>145</v>
       </c>
@@ -3661,12 +3661,12 @@
       <c r="H93" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I93" s="18"/>
-      <c r="J93" s="19"/>
-      <c r="K93" s="18"/>
+      <c r="I93" s="15"/>
+      <c r="J93" s="16"/>
+      <c r="K93" s="15"/>
     </row>
     <row r="94" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B94" s="17"/>
+      <c r="B94" s="14"/>
       <c r="C94" s="7" t="s">
         <v>146</v>
       </c>
@@ -3685,12 +3685,12 @@
       <c r="H94" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I94" s="18"/>
-      <c r="J94" s="19"/>
-      <c r="K94" s="18"/>
+      <c r="I94" s="15"/>
+      <c r="J94" s="16"/>
+      <c r="K94" s="15"/>
     </row>
     <row r="95" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B95" s="17"/>
+      <c r="B95" s="14"/>
       <c r="C95" s="7" t="s">
         <v>147</v>
       </c>
@@ -3709,12 +3709,12 @@
       <c r="H95" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I95" s="18"/>
-      <c r="J95" s="19"/>
-      <c r="K95" s="18"/>
+      <c r="I95" s="15"/>
+      <c r="J95" s="16"/>
+      <c r="K95" s="15"/>
     </row>
     <row r="96" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B96" s="17"/>
+      <c r="B96" s="14"/>
       <c r="C96" s="7" t="s">
         <v>148</v>
       </c>
@@ -3733,28 +3733,28 @@
       <c r="H96" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I96" s="18"/>
-      <c r="J96" s="19"/>
-      <c r="K96" s="18"/>
+      <c r="I96" s="15"/>
+      <c r="J96" s="16"/>
+      <c r="K96" s="15"/>
     </row>
     <row r="97" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B97" s="17" t="s">
+      <c r="B97" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="C97" s="15" t="s">
+      <c r="C97" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="D97" s="15"/>
-      <c r="E97" s="15"/>
-      <c r="F97" s="15"/>
-      <c r="G97" s="15"/>
-      <c r="H97" s="15"/>
-      <c r="I97" s="15"/>
-      <c r="J97" s="15"/>
-      <c r="K97" s="15"/>
+      <c r="D97" s="13"/>
+      <c r="E97" s="13"/>
+      <c r="F97" s="13"/>
+      <c r="G97" s="13"/>
+      <c r="H97" s="13"/>
+      <c r="I97" s="13"/>
+      <c r="J97" s="13"/>
+      <c r="K97" s="13"/>
     </row>
     <row r="98" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B98" s="17"/>
+      <c r="B98" s="14"/>
       <c r="C98" s="7" t="s">
         <v>158</v>
       </c>
@@ -3773,18 +3773,18 @@
       <c r="H98" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I98" s="18" t="s">
+      <c r="I98" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="J98" s="19" t="s">
+      <c r="J98" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K98" s="18" t="s">
+      <c r="K98" s="15" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="99" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B99" s="17"/>
+      <c r="B99" s="14"/>
       <c r="C99" s="7" t="s">
         <v>159</v>
       </c>
@@ -3803,12 +3803,12 @@
       <c r="H99" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I99" s="18"/>
-      <c r="J99" s="19"/>
-      <c r="K99" s="18"/>
+      <c r="I99" s="15"/>
+      <c r="J99" s="16"/>
+      <c r="K99" s="15"/>
     </row>
     <row r="100" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B100" s="17"/>
+      <c r="B100" s="14"/>
       <c r="C100" s="7" t="s">
         <v>160</v>
       </c>
@@ -3827,12 +3827,12 @@
       <c r="H100" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I100" s="18"/>
-      <c r="J100" s="19"/>
-      <c r="K100" s="18"/>
+      <c r="I100" s="15"/>
+      <c r="J100" s="16"/>
+      <c r="K100" s="15"/>
     </row>
     <row r="101" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B101" s="17"/>
+      <c r="B101" s="14"/>
       <c r="C101" s="7" t="s">
         <v>161</v>
       </c>
@@ -3851,12 +3851,12 @@
       <c r="H101" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I101" s="18"/>
-      <c r="J101" s="19"/>
-      <c r="K101" s="18"/>
+      <c r="I101" s="15"/>
+      <c r="J101" s="16"/>
+      <c r="K101" s="15"/>
     </row>
     <row r="102" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B102" s="17"/>
+      <c r="B102" s="14"/>
       <c r="C102" s="7" t="s">
         <v>162</v>
       </c>
@@ -3875,12 +3875,12 @@
       <c r="H102" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I102" s="18"/>
-      <c r="J102" s="19"/>
-      <c r="K102" s="18"/>
+      <c r="I102" s="15"/>
+      <c r="J102" s="16"/>
+      <c r="K102" s="15"/>
     </row>
     <row r="103" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B103" s="17"/>
+      <c r="B103" s="14"/>
       <c r="C103" s="7" t="s">
         <v>163</v>
       </c>
@@ -3899,12 +3899,12 @@
       <c r="H103" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I103" s="18"/>
-      <c r="J103" s="19"/>
-      <c r="K103" s="18"/>
+      <c r="I103" s="15"/>
+      <c r="J103" s="16"/>
+      <c r="K103" s="15"/>
     </row>
     <row r="104" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B104" s="17"/>
+      <c r="B104" s="14"/>
       <c r="C104" s="7" t="s">
         <v>164</v>
       </c>
@@ -3923,12 +3923,12 @@
       <c r="H104" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I104" s="18"/>
-      <c r="J104" s="19"/>
-      <c r="K104" s="18"/>
+      <c r="I104" s="15"/>
+      <c r="J104" s="16"/>
+      <c r="K104" s="15"/>
     </row>
     <row r="105" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B105" s="17"/>
+      <c r="B105" s="14"/>
       <c r="C105" s="7" t="s">
         <v>165</v>
       </c>
@@ -3947,12 +3947,12 @@
       <c r="H105" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I105" s="18"/>
-      <c r="J105" s="19"/>
-      <c r="K105" s="18"/>
+      <c r="I105" s="15"/>
+      <c r="J105" s="16"/>
+      <c r="K105" s="15"/>
     </row>
     <row r="106" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B106" s="17"/>
+      <c r="B106" s="14"/>
       <c r="C106" s="7" t="s">
         <v>166</v>
       </c>
@@ -3971,12 +3971,12 @@
       <c r="H106" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I106" s="18"/>
-      <c r="J106" s="19"/>
-      <c r="K106" s="18"/>
+      <c r="I106" s="15"/>
+      <c r="J106" s="16"/>
+      <c r="K106" s="15"/>
     </row>
     <row r="107" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B107" s="17"/>
+      <c r="B107" s="14"/>
       <c r="C107" s="7" t="s">
         <v>167</v>
       </c>
@@ -3995,12 +3995,12 @@
       <c r="H107" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I107" s="18"/>
-      <c r="J107" s="19"/>
-      <c r="K107" s="18"/>
+      <c r="I107" s="15"/>
+      <c r="J107" s="16"/>
+      <c r="K107" s="15"/>
     </row>
     <row r="108" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B108" s="17"/>
+      <c r="B108" s="14"/>
       <c r="C108" s="7" t="s">
         <v>168</v>
       </c>
@@ -4019,12 +4019,12 @@
       <c r="H108" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I108" s="18"/>
-      <c r="J108" s="19"/>
-      <c r="K108" s="18"/>
+      <c r="I108" s="15"/>
+      <c r="J108" s="16"/>
+      <c r="K108" s="15"/>
     </row>
     <row r="109" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B109" s="17"/>
+      <c r="B109" s="14"/>
       <c r="C109" s="7" t="s">
         <v>169</v>
       </c>
@@ -4043,12 +4043,12 @@
       <c r="H109" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I109" s="18"/>
-      <c r="J109" s="19"/>
-      <c r="K109" s="18"/>
+      <c r="I109" s="15"/>
+      <c r="J109" s="16"/>
+      <c r="K109" s="15"/>
     </row>
     <row r="110" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B110" s="17"/>
+      <c r="B110" s="14"/>
       <c r="C110" s="7" t="s">
         <v>170</v>
       </c>
@@ -4067,28 +4067,28 @@
       <c r="H110" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I110" s="18"/>
-      <c r="J110" s="19"/>
-      <c r="K110" s="18"/>
+      <c r="I110" s="15"/>
+      <c r="J110" s="16"/>
+      <c r="K110" s="15"/>
     </row>
     <row r="111" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B111" s="17" t="s">
+      <c r="B111" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="C111" s="15" t="s">
+      <c r="C111" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="D111" s="15"/>
-      <c r="E111" s="15"/>
-      <c r="F111" s="15"/>
-      <c r="G111" s="15"/>
-      <c r="H111" s="15"/>
-      <c r="I111" s="15"/>
-      <c r="J111" s="15"/>
-      <c r="K111" s="15"/>
+      <c r="D111" s="13"/>
+      <c r="E111" s="13"/>
+      <c r="F111" s="13"/>
+      <c r="G111" s="13"/>
+      <c r="H111" s="13"/>
+      <c r="I111" s="13"/>
+      <c r="J111" s="13"/>
+      <c r="K111" s="13"/>
     </row>
     <row r="112" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B112" s="17"/>
+      <c r="B112" s="14"/>
       <c r="C112" s="7" t="s">
         <v>175</v>
       </c>
@@ -4107,18 +4107,18 @@
       <c r="H112" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I112" s="18" t="s">
+      <c r="I112" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="J112" s="19" t="s">
+      <c r="J112" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K112" s="18" t="s">
+      <c r="K112" s="15" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="113" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B113" s="17"/>
+      <c r="B113" s="14"/>
       <c r="C113" s="7" t="s">
         <v>176</v>
       </c>
@@ -4137,12 +4137,12 @@
       <c r="H113" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I113" s="18"/>
-      <c r="J113" s="19"/>
-      <c r="K113" s="18"/>
+      <c r="I113" s="15"/>
+      <c r="J113" s="16"/>
+      <c r="K113" s="15"/>
     </row>
     <row r="114" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B114" s="17"/>
+      <c r="B114" s="14"/>
       <c r="C114" s="7" t="s">
         <v>177</v>
       </c>
@@ -4161,12 +4161,12 @@
       <c r="H114" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I114" s="18"/>
-      <c r="J114" s="19"/>
-      <c r="K114" s="18"/>
+      <c r="I114" s="15"/>
+      <c r="J114" s="16"/>
+      <c r="K114" s="15"/>
     </row>
     <row r="115" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B115" s="17"/>
+      <c r="B115" s="14"/>
       <c r="C115" s="7" t="s">
         <v>178</v>
       </c>
@@ -4185,12 +4185,12 @@
       <c r="H115" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I115" s="18"/>
-      <c r="J115" s="19"/>
-      <c r="K115" s="18"/>
+      <c r="I115" s="15"/>
+      <c r="J115" s="16"/>
+      <c r="K115" s="15"/>
     </row>
     <row r="116" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B116" s="17"/>
+      <c r="B116" s="14"/>
       <c r="C116" s="7" t="s">
         <v>179</v>
       </c>
@@ -4209,12 +4209,12 @@
       <c r="H116" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I116" s="18"/>
-      <c r="J116" s="19"/>
-      <c r="K116" s="18"/>
+      <c r="I116" s="15"/>
+      <c r="J116" s="16"/>
+      <c r="K116" s="15"/>
     </row>
     <row r="117" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B117" s="17"/>
+      <c r="B117" s="14"/>
       <c r="C117" s="7" t="s">
         <v>180</v>
       </c>
@@ -4233,12 +4233,12 @@
       <c r="H117" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I117" s="18"/>
-      <c r="J117" s="19"/>
-      <c r="K117" s="18"/>
+      <c r="I117" s="15"/>
+      <c r="J117" s="16"/>
+      <c r="K117" s="15"/>
     </row>
     <row r="118" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B118" s="17"/>
+      <c r="B118" s="14"/>
       <c r="C118" s="7" t="s">
         <v>181</v>
       </c>
@@ -4257,12 +4257,12 @@
       <c r="H118" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I118" s="18"/>
-      <c r="J118" s="19"/>
-      <c r="K118" s="18"/>
+      <c r="I118" s="15"/>
+      <c r="J118" s="16"/>
+      <c r="K118" s="15"/>
     </row>
     <row r="119" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B119" s="17"/>
+      <c r="B119" s="14"/>
       <c r="C119" s="7" t="s">
         <v>182</v>
       </c>
@@ -4281,28 +4281,28 @@
       <c r="H119" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I119" s="18"/>
-      <c r="J119" s="19"/>
-      <c r="K119" s="18"/>
+      <c r="I119" s="15"/>
+      <c r="J119" s="16"/>
+      <c r="K119" s="15"/>
     </row>
     <row r="120" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B120" s="17" t="s">
+      <c r="B120" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="C120" s="15" t="s">
+      <c r="C120" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="D120" s="15"/>
-      <c r="E120" s="15"/>
-      <c r="F120" s="15"/>
-      <c r="G120" s="15"/>
-      <c r="H120" s="15"/>
-      <c r="I120" s="15"/>
-      <c r="J120" s="15"/>
-      <c r="K120" s="15"/>
+      <c r="D120" s="13"/>
+      <c r="E120" s="13"/>
+      <c r="F120" s="13"/>
+      <c r="G120" s="13"/>
+      <c r="H120" s="13"/>
+      <c r="I120" s="13"/>
+      <c r="J120" s="13"/>
+      <c r="K120" s="13"/>
     </row>
     <row r="121" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B121" s="17"/>
+      <c r="B121" s="14"/>
       <c r="C121" s="7" t="s">
         <v>187</v>
       </c>
@@ -4321,18 +4321,18 @@
       <c r="H121" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I121" s="18" t="s">
+      <c r="I121" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="J121" s="19" t="s">
+      <c r="J121" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K121" s="18" t="s">
+      <c r="K121" s="15" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="122" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B122" s="17"/>
+      <c r="B122" s="14"/>
       <c r="C122" s="7" t="s">
         <v>188</v>
       </c>
@@ -4351,12 +4351,12 @@
       <c r="H122" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I122" s="18"/>
-      <c r="J122" s="19"/>
-      <c r="K122" s="18"/>
+      <c r="I122" s="15"/>
+      <c r="J122" s="16"/>
+      <c r="K122" s="15"/>
     </row>
     <row r="123" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B123" s="17"/>
+      <c r="B123" s="14"/>
       <c r="C123" s="7" t="s">
         <v>189</v>
       </c>
@@ -4375,12 +4375,12 @@
       <c r="H123" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I123" s="18"/>
-      <c r="J123" s="19"/>
-      <c r="K123" s="18"/>
+      <c r="I123" s="15"/>
+      <c r="J123" s="16"/>
+      <c r="K123" s="15"/>
     </row>
     <row r="124" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B124" s="17"/>
+      <c r="B124" s="14"/>
       <c r="C124" s="7" t="s">
         <v>190</v>
       </c>
@@ -4399,12 +4399,12 @@
       <c r="H124" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I124" s="18"/>
-      <c r="J124" s="19"/>
-      <c r="K124" s="18"/>
+      <c r="I124" s="15"/>
+      <c r="J124" s="16"/>
+      <c r="K124" s="15"/>
     </row>
     <row r="125" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B125" s="17"/>
+      <c r="B125" s="14"/>
       <c r="C125" s="7" t="s">
         <v>191</v>
       </c>
@@ -4423,12 +4423,12 @@
       <c r="H125" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I125" s="18"/>
-      <c r="J125" s="19"/>
-      <c r="K125" s="18"/>
+      <c r="I125" s="15"/>
+      <c r="J125" s="16"/>
+      <c r="K125" s="15"/>
     </row>
     <row r="126" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B126" s="17"/>
+      <c r="B126" s="14"/>
       <c r="C126" s="7" t="s">
         <v>192</v>
       </c>
@@ -4447,28 +4447,28 @@
       <c r="H126" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I126" s="18"/>
-      <c r="J126" s="19"/>
-      <c r="K126" s="18"/>
+      <c r="I126" s="15"/>
+      <c r="J126" s="16"/>
+      <c r="K126" s="15"/>
     </row>
     <row r="127" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B127" s="17" t="s">
+      <c r="B127" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="C127" s="15" t="s">
+      <c r="C127" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="D127" s="15"/>
-      <c r="E127" s="15"/>
-      <c r="F127" s="15"/>
-      <c r="G127" s="15"/>
-      <c r="H127" s="15"/>
-      <c r="I127" s="15"/>
-      <c r="J127" s="15"/>
-      <c r="K127" s="15"/>
+      <c r="D127" s="13"/>
+      <c r="E127" s="13"/>
+      <c r="F127" s="13"/>
+      <c r="G127" s="13"/>
+      <c r="H127" s="13"/>
+      <c r="I127" s="13"/>
+      <c r="J127" s="13"/>
+      <c r="K127" s="13"/>
     </row>
     <row r="128" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B128" s="17"/>
+      <c r="B128" s="14"/>
       <c r="C128" s="7" t="s">
         <v>197</v>
       </c>
@@ -4487,18 +4487,18 @@
       <c r="H128" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I128" s="18" t="s">
+      <c r="I128" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="J128" s="19" t="s">
+      <c r="J128" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K128" s="18" t="s">
+      <c r="K128" s="15" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="129" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B129" s="17"/>
+      <c r="B129" s="14"/>
       <c r="C129" s="7" t="s">
         <v>198</v>
       </c>
@@ -4517,12 +4517,12 @@
       <c r="H129" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I129" s="18"/>
-      <c r="J129" s="19"/>
-      <c r="K129" s="18"/>
+      <c r="I129" s="15"/>
+      <c r="J129" s="16"/>
+      <c r="K129" s="15"/>
     </row>
     <row r="130" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B130" s="17"/>
+      <c r="B130" s="14"/>
       <c r="C130" s="7" t="s">
         <v>199</v>
       </c>
@@ -4541,12 +4541,12 @@
       <c r="H130" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I130" s="18"/>
-      <c r="J130" s="19"/>
-      <c r="K130" s="18"/>
+      <c r="I130" s="15"/>
+      <c r="J130" s="16"/>
+      <c r="K130" s="15"/>
     </row>
     <row r="131" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B131" s="17"/>
+      <c r="B131" s="14"/>
       <c r="C131" s="7" t="s">
         <v>200</v>
       </c>
@@ -4565,12 +4565,12 @@
       <c r="H131" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I131" s="18"/>
-      <c r="J131" s="19"/>
-      <c r="K131" s="18"/>
+      <c r="I131" s="15"/>
+      <c r="J131" s="16"/>
+      <c r="K131" s="15"/>
     </row>
     <row r="132" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B132" s="17"/>
+      <c r="B132" s="14"/>
       <c r="C132" s="7" t="s">
         <v>201</v>
       </c>
@@ -4589,12 +4589,12 @@
       <c r="H132" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I132" s="18"/>
-      <c r="J132" s="19"/>
-      <c r="K132" s="18"/>
+      <c r="I132" s="15"/>
+      <c r="J132" s="16"/>
+      <c r="K132" s="15"/>
     </row>
     <row r="133" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B133" s="17"/>
+      <c r="B133" s="14"/>
       <c r="C133" s="7" t="s">
         <v>202</v>
       </c>
@@ -4613,12 +4613,12 @@
       <c r="H133" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I133" s="18"/>
-      <c r="J133" s="19"/>
-      <c r="K133" s="18"/>
+      <c r="I133" s="15"/>
+      <c r="J133" s="16"/>
+      <c r="K133" s="15"/>
     </row>
     <row r="134" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B134" s="17"/>
+      <c r="B134" s="14"/>
       <c r="C134" s="7" t="s">
         <v>203</v>
       </c>
@@ -4637,29 +4637,29 @@
       <c r="H134" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I134" s="18"/>
-      <c r="J134" s="19"/>
-      <c r="K134" s="18"/>
+      <c r="I134" s="15"/>
+      <c r="J134" s="16"/>
+      <c r="K134" s="15"/>
     </row>
     <row r="135" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B135" s="17" t="s">
+      <c r="B135" s="14" t="s">
         <v>213</v>
       </c>
-      <c r="C135" s="20" t="s">
+      <c r="C135" s="12" t="s">
         <v>208</v>
       </c>
-      <c r="D135" s="15"/>
-      <c r="E135" s="15"/>
-      <c r="F135" s="15"/>
-      <c r="G135" s="15"/>
-      <c r="H135" s="15"/>
-      <c r="I135" s="15"/>
-      <c r="J135" s="15"/>
-      <c r="K135" s="15"/>
+      <c r="D135" s="13"/>
+      <c r="E135" s="13"/>
+      <c r="F135" s="13"/>
+      <c r="G135" s="13"/>
+      <c r="H135" s="13"/>
+      <c r="I135" s="13"/>
+      <c r="J135" s="13"/>
+      <c r="K135" s="13"/>
     </row>
     <row r="136" spans="2:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B136" s="17"/>
-      <c r="C136" s="21" t="s">
+      <c r="B136" s="14"/>
+      <c r="C136" s="11" t="s">
         <v>214</v>
       </c>
       <c r="D136" s="8" t="s">
@@ -4677,19 +4677,19 @@
       <c r="H136" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I136" s="18" t="s">
+      <c r="I136" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="J136" s="19" t="s">
+      <c r="J136" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K136" s="18" t="s">
+      <c r="K136" s="15" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="137" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B137" s="17"/>
-      <c r="C137" s="21" t="s">
+      <c r="B137" s="14"/>
+      <c r="C137" s="11" t="s">
         <v>215</v>
       </c>
       <c r="D137" s="3" t="s">
@@ -4707,13 +4707,13 @@
       <c r="H137" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I137" s="18"/>
-      <c r="J137" s="19"/>
-      <c r="K137" s="18"/>
+      <c r="I137" s="15"/>
+      <c r="J137" s="16"/>
+      <c r="K137" s="15"/>
     </row>
     <row r="138" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B138" s="17"/>
-      <c r="C138" s="21" t="s">
+      <c r="B138" s="14"/>
+      <c r="C138" s="11" t="s">
         <v>216</v>
       </c>
       <c r="D138" s="3" t="s">
@@ -4731,13 +4731,13 @@
       <c r="H138" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I138" s="18"/>
-      <c r="J138" s="19"/>
-      <c r="K138" s="18"/>
+      <c r="I138" s="15"/>
+      <c r="J138" s="16"/>
+      <c r="K138" s="15"/>
     </row>
     <row r="139" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B139" s="17"/>
-      <c r="C139" s="21" t="s">
+      <c r="B139" s="14"/>
+      <c r="C139" s="11" t="s">
         <v>217</v>
       </c>
       <c r="D139" s="3" t="s">
@@ -4755,13 +4755,13 @@
       <c r="H139" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I139" s="18"/>
-      <c r="J139" s="19"/>
-      <c r="K139" s="18"/>
+      <c r="I139" s="15"/>
+      <c r="J139" s="16"/>
+      <c r="K139" s="15"/>
     </row>
     <row r="140" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B140" s="17"/>
-      <c r="C140" s="21" t="s">
+      <c r="B140" s="14"/>
+      <c r="C140" s="11" t="s">
         <v>218</v>
       </c>
       <c r="D140" s="3" t="s">
@@ -4779,13 +4779,13 @@
       <c r="H140" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I140" s="18"/>
-      <c r="J140" s="19"/>
-      <c r="K140" s="18"/>
+      <c r="I140" s="15"/>
+      <c r="J140" s="16"/>
+      <c r="K140" s="15"/>
     </row>
     <row r="141" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B141" s="17"/>
-      <c r="C141" s="21" t="s">
+      <c r="B141" s="14"/>
+      <c r="C141" s="11" t="s">
         <v>219</v>
       </c>
       <c r="D141" s="3" t="s">
@@ -4803,13 +4803,13 @@
       <c r="H141" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I141" s="18"/>
-      <c r="J141" s="19"/>
-      <c r="K141" s="18"/>
+      <c r="I141" s="15"/>
+      <c r="J141" s="16"/>
+      <c r="K141" s="15"/>
     </row>
     <row r="142" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B142" s="17"/>
-      <c r="C142" s="21" t="s">
+      <c r="B142" s="14"/>
+      <c r="C142" s="11" t="s">
         <v>220</v>
       </c>
       <c r="D142" s="3" t="s">
@@ -4827,13 +4827,13 @@
       <c r="H142" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I142" s="18"/>
-      <c r="J142" s="19"/>
-      <c r="K142" s="18"/>
+      <c r="I142" s="15"/>
+      <c r="J142" s="16"/>
+      <c r="K142" s="15"/>
     </row>
     <row r="143" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B143" s="17"/>
-      <c r="C143" s="21" t="s">
+      <c r="B143" s="14"/>
+      <c r="C143" s="11" t="s">
         <v>221</v>
       </c>
       <c r="D143" s="3" t="s">
@@ -4851,13 +4851,13 @@
       <c r="H143" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I143" s="18"/>
-      <c r="J143" s="19"/>
-      <c r="K143" s="18"/>
+      <c r="I143" s="15"/>
+      <c r="J143" s="16"/>
+      <c r="K143" s="15"/>
     </row>
     <row r="144" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B144" s="17"/>
-      <c r="C144" s="21" t="s">
+      <c r="B144" s="14"/>
+      <c r="C144" s="11" t="s">
         <v>222</v>
       </c>
       <c r="D144" s="3" t="s">
@@ -4875,13 +4875,13 @@
       <c r="H144" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I144" s="18"/>
-      <c r="J144" s="19"/>
-      <c r="K144" s="18"/>
+      <c r="I144" s="15"/>
+      <c r="J144" s="16"/>
+      <c r="K144" s="15"/>
     </row>
     <row r="145" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B145" s="17"/>
-      <c r="C145" s="21" t="s">
+      <c r="B145" s="14"/>
+      <c r="C145" s="11" t="s">
         <v>223</v>
       </c>
       <c r="D145" s="3" t="s">
@@ -4899,13 +4899,13 @@
       <c r="H145" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I145" s="18"/>
-      <c r="J145" s="19"/>
-      <c r="K145" s="18"/>
+      <c r="I145" s="15"/>
+      <c r="J145" s="16"/>
+      <c r="K145" s="15"/>
     </row>
     <row r="146" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B146" s="17"/>
-      <c r="C146" s="21" t="s">
+      <c r="B146" s="14"/>
+      <c r="C146" s="11" t="s">
         <v>224</v>
       </c>
       <c r="D146" s="3" t="s">
@@ -4923,13 +4923,13 @@
       <c r="H146" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I146" s="18"/>
-      <c r="J146" s="19"/>
-      <c r="K146" s="18"/>
+      <c r="I146" s="15"/>
+      <c r="J146" s="16"/>
+      <c r="K146" s="15"/>
     </row>
     <row r="147" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B147" s="17"/>
-      <c r="C147" s="21" t="s">
+      <c r="B147" s="14"/>
+      <c r="C147" s="11" t="s">
         <v>225</v>
       </c>
       <c r="D147" s="3" t="s">
@@ -4947,13 +4947,13 @@
       <c r="H147" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I147" s="18"/>
-      <c r="J147" s="19"/>
-      <c r="K147" s="18"/>
+      <c r="I147" s="15"/>
+      <c r="J147" s="16"/>
+      <c r="K147" s="15"/>
     </row>
     <row r="148" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B148" s="17"/>
-      <c r="C148" s="21" t="s">
+      <c r="B148" s="14"/>
+      <c r="C148" s="11" t="s">
         <v>226</v>
       </c>
       <c r="D148" s="3" t="s">
@@ -4971,13 +4971,13 @@
       <c r="H148" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I148" s="18"/>
-      <c r="J148" s="19"/>
-      <c r="K148" s="18"/>
+      <c r="I148" s="15"/>
+      <c r="J148" s="16"/>
+      <c r="K148" s="15"/>
     </row>
     <row r="149" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B149" s="17"/>
-      <c r="C149" s="21" t="s">
+      <c r="B149" s="14"/>
+      <c r="C149" s="11" t="s">
         <v>227</v>
       </c>
       <c r="D149" s="3" t="s">
@@ -4995,13 +4995,13 @@
       <c r="H149" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I149" s="18"/>
-      <c r="J149" s="19"/>
-      <c r="K149" s="18"/>
+      <c r="I149" s="15"/>
+      <c r="J149" s="16"/>
+      <c r="K149" s="15"/>
     </row>
     <row r="150" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B150" s="17"/>
-      <c r="C150" s="21" t="s">
+      <c r="B150" s="14"/>
+      <c r="C150" s="11" t="s">
         <v>228</v>
       </c>
       <c r="D150" s="3" t="s">
@@ -5019,13 +5019,13 @@
       <c r="H150" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I150" s="18"/>
-      <c r="J150" s="19"/>
-      <c r="K150" s="18"/>
+      <c r="I150" s="15"/>
+      <c r="J150" s="16"/>
+      <c r="K150" s="15"/>
     </row>
     <row r="151" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B151" s="17"/>
-      <c r="C151" s="21" t="s">
+      <c r="B151" s="14"/>
+      <c r="C151" s="11" t="s">
         <v>229</v>
       </c>
       <c r="D151" s="3" t="s">
@@ -5043,13 +5043,13 @@
       <c r="H151" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I151" s="18"/>
-      <c r="J151" s="19"/>
-      <c r="K151" s="18"/>
+      <c r="I151" s="15"/>
+      <c r="J151" s="16"/>
+      <c r="K151" s="15"/>
     </row>
     <row r="152" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B152" s="17"/>
-      <c r="C152" s="21" t="s">
+      <c r="B152" s="14"/>
+      <c r="C152" s="11" t="s">
         <v>230</v>
       </c>
       <c r="D152" s="3" t="s">
@@ -5067,13 +5067,13 @@
       <c r="H152" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I152" s="18"/>
-      <c r="J152" s="19"/>
-      <c r="K152" s="18"/>
+      <c r="I152" s="15"/>
+      <c r="J152" s="16"/>
+      <c r="K152" s="15"/>
     </row>
     <row r="153" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B153" s="17"/>
-      <c r="C153" s="21" t="s">
+      <c r="B153" s="14"/>
+      <c r="C153" s="11" t="s">
         <v>231</v>
       </c>
       <c r="D153" s="3" t="s">
@@ -5091,13 +5091,13 @@
       <c r="H153" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I153" s="18"/>
-      <c r="J153" s="19"/>
-      <c r="K153" s="18"/>
+      <c r="I153" s="15"/>
+      <c r="J153" s="16"/>
+      <c r="K153" s="15"/>
     </row>
     <row r="154" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B154" s="17"/>
-      <c r="C154" s="21" t="s">
+      <c r="B154" s="14"/>
+      <c r="C154" s="11" t="s">
         <v>232</v>
       </c>
       <c r="D154" s="3" t="s">
@@ -5115,13 +5115,13 @@
       <c r="H154" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I154" s="18"/>
-      <c r="J154" s="19"/>
-      <c r="K154" s="18"/>
+      <c r="I154" s="15"/>
+      <c r="J154" s="16"/>
+      <c r="K154" s="15"/>
     </row>
     <row r="155" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B155" s="17"/>
-      <c r="C155" s="21" t="s">
+      <c r="B155" s="14"/>
+      <c r="C155" s="11" t="s">
         <v>233</v>
       </c>
       <c r="D155" s="3" t="s">
@@ -5139,29 +5139,29 @@
       <c r="H155" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I155" s="18"/>
-      <c r="J155" s="19"/>
-      <c r="K155" s="18"/>
+      <c r="I155" s="15"/>
+      <c r="J155" s="16"/>
+      <c r="K155" s="15"/>
     </row>
     <row r="156" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B156" s="17" t="s">
+      <c r="B156" s="14" t="s">
         <v>242</v>
       </c>
-      <c r="C156" s="20" t="s">
+      <c r="C156" s="12" t="s">
         <v>234</v>
       </c>
-      <c r="D156" s="15"/>
-      <c r="E156" s="15"/>
-      <c r="F156" s="15"/>
-      <c r="G156" s="15"/>
-      <c r="H156" s="15"/>
-      <c r="I156" s="15"/>
-      <c r="J156" s="15"/>
-      <c r="K156" s="15"/>
+      <c r="D156" s="13"/>
+      <c r="E156" s="13"/>
+      <c r="F156" s="13"/>
+      <c r="G156" s="13"/>
+      <c r="H156" s="13"/>
+      <c r="I156" s="13"/>
+      <c r="J156" s="13"/>
+      <c r="K156" s="13"/>
     </row>
     <row r="157" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B157" s="17"/>
-      <c r="C157" s="21" t="s">
+      <c r="B157" s="14"/>
+      <c r="C157" s="11" t="s">
         <v>243</v>
       </c>
       <c r="D157" s="8" t="s">
@@ -5179,17 +5179,17 @@
       <c r="H157" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I157" s="18" t="s">
+      <c r="I157" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="J157" s="19" t="s">
+      <c r="J157" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K157" s="18"/>
+      <c r="K157" s="15"/>
     </row>
     <row r="158" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B158" s="17"/>
-      <c r="C158" s="21" t="s">
+      <c r="B158" s="14"/>
+      <c r="C158" s="11" t="s">
         <v>244</v>
       </c>
       <c r="D158" s="3" t="s">
@@ -5207,13 +5207,13 @@
       <c r="H158" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I158" s="18"/>
-      <c r="J158" s="19"/>
-      <c r="K158" s="18"/>
+      <c r="I158" s="15"/>
+      <c r="J158" s="16"/>
+      <c r="K158" s="15"/>
     </row>
     <row r="159" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B159" s="17"/>
-      <c r="C159" s="21" t="s">
+      <c r="B159" s="14"/>
+      <c r="C159" s="11" t="s">
         <v>245</v>
       </c>
       <c r="D159" s="3" t="s">
@@ -5231,13 +5231,13 @@
       <c r="H159" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I159" s="18"/>
-      <c r="J159" s="19"/>
-      <c r="K159" s="18"/>
+      <c r="I159" s="15"/>
+      <c r="J159" s="16"/>
+      <c r="K159" s="15"/>
     </row>
     <row r="160" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B160" s="17"/>
-      <c r="C160" s="21" t="s">
+      <c r="B160" s="14"/>
+      <c r="C160" s="11" t="s">
         <v>246</v>
       </c>
       <c r="D160" s="3" t="s">
@@ -5255,13 +5255,13 @@
       <c r="H160" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I160" s="18"/>
-      <c r="J160" s="19"/>
-      <c r="K160" s="18"/>
+      <c r="I160" s="15"/>
+      <c r="J160" s="16"/>
+      <c r="K160" s="15"/>
     </row>
     <row r="161" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B161" s="17"/>
-      <c r="C161" s="21" t="s">
+      <c r="B161" s="14"/>
+      <c r="C161" s="11" t="s">
         <v>247</v>
       </c>
       <c r="D161" s="3" t="s">
@@ -5279,13 +5279,13 @@
       <c r="H161" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I161" s="18"/>
-      <c r="J161" s="19"/>
-      <c r="K161" s="18"/>
+      <c r="I161" s="15"/>
+      <c r="J161" s="16"/>
+      <c r="K161" s="15"/>
     </row>
     <row r="162" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B162" s="17"/>
-      <c r="C162" s="21" t="s">
+      <c r="B162" s="14"/>
+      <c r="C162" s="11" t="s">
         <v>248</v>
       </c>
       <c r="D162" s="3" t="s">
@@ -5303,13 +5303,13 @@
       <c r="H162" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I162" s="18"/>
-      <c r="J162" s="19"/>
-      <c r="K162" s="18"/>
+      <c r="I162" s="15"/>
+      <c r="J162" s="16"/>
+      <c r="K162" s="15"/>
     </row>
     <row r="163" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B163" s="17"/>
-      <c r="C163" s="21" t="s">
+      <c r="B163" s="14"/>
+      <c r="C163" s="11" t="s">
         <v>249</v>
       </c>
       <c r="D163" s="3" t="s">
@@ -5327,13 +5327,13 @@
       <c r="H163" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I163" s="18"/>
-      <c r="J163" s="19"/>
-      <c r="K163" s="18"/>
+      <c r="I163" s="15"/>
+      <c r="J163" s="16"/>
+      <c r="K163" s="15"/>
     </row>
     <row r="164" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B164" s="17"/>
-      <c r="C164" s="21" t="s">
+      <c r="B164" s="14"/>
+      <c r="C164" s="11" t="s">
         <v>250</v>
       </c>
       <c r="D164" s="3" t="s">
@@ -5351,13 +5351,13 @@
       <c r="H164" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I164" s="18"/>
-      <c r="J164" s="19"/>
-      <c r="K164" s="18"/>
+      <c r="I164" s="15"/>
+      <c r="J164" s="16"/>
+      <c r="K164" s="15"/>
     </row>
     <row r="165" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B165" s="17"/>
-      <c r="C165" s="21" t="s">
+      <c r="B165" s="14"/>
+      <c r="C165" s="11" t="s">
         <v>251</v>
       </c>
       <c r="D165" s="3" t="s">
@@ -5375,29 +5375,29 @@
       <c r="H165" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I165" s="18"/>
-      <c r="J165" s="19"/>
-      <c r="K165" s="18"/>
+      <c r="I165" s="15"/>
+      <c r="J165" s="16"/>
+      <c r="K165" s="15"/>
     </row>
     <row r="166" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B166" s="17" t="s">
+      <c r="B166" s="14" t="s">
         <v>253</v>
       </c>
-      <c r="C166" s="20" t="s">
+      <c r="C166" s="12" t="s">
         <v>252</v>
       </c>
-      <c r="D166" s="15"/>
-      <c r="E166" s="15"/>
-      <c r="F166" s="15"/>
-      <c r="G166" s="15"/>
-      <c r="H166" s="15"/>
-      <c r="I166" s="15"/>
-      <c r="J166" s="15"/>
-      <c r="K166" s="15"/>
+      <c r="D166" s="13"/>
+      <c r="E166" s="13"/>
+      <c r="F166" s="13"/>
+      <c r="G166" s="13"/>
+      <c r="H166" s="13"/>
+      <c r="I166" s="13"/>
+      <c r="J166" s="13"/>
+      <c r="K166" s="13"/>
     </row>
     <row r="167" spans="2:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B167" s="17"/>
-      <c r="C167" s="21" t="s">
+      <c r="B167" s="14"/>
+      <c r="C167" s="11" t="s">
         <v>267</v>
       </c>
       <c r="D167" s="8" t="s">
@@ -5415,17 +5415,17 @@
       <c r="H167" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I167" s="18" t="s">
+      <c r="I167" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="J167" s="19" t="s">
+      <c r="J167" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K167" s="18"/>
+      <c r="K167" s="15"/>
     </row>
     <row r="168" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B168" s="17"/>
-      <c r="C168" s="21" t="s">
+      <c r="B168" s="14"/>
+      <c r="C168" s="11" t="s">
         <v>268</v>
       </c>
       <c r="D168" s="3" t="s">
@@ -5443,13 +5443,13 @@
       <c r="H168" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I168" s="18"/>
-      <c r="J168" s="19"/>
-      <c r="K168" s="18"/>
+      <c r="I168" s="15"/>
+      <c r="J168" s="16"/>
+      <c r="K168" s="15"/>
     </row>
     <row r="169" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B169" s="17"/>
-      <c r="C169" s="21" t="s">
+      <c r="B169" s="14"/>
+      <c r="C169" s="11" t="s">
         <v>269</v>
       </c>
       <c r="D169" s="3" t="s">
@@ -5467,13 +5467,13 @@
       <c r="H169" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I169" s="18"/>
-      <c r="J169" s="19"/>
-      <c r="K169" s="18"/>
+      <c r="I169" s="15"/>
+      <c r="J169" s="16"/>
+      <c r="K169" s="15"/>
     </row>
     <row r="170" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B170" s="17"/>
-      <c r="C170" s="21" t="s">
+      <c r="B170" s="14"/>
+      <c r="C170" s="11" t="s">
         <v>270</v>
       </c>
       <c r="D170" s="3" t="s">
@@ -5491,13 +5491,13 @@
       <c r="H170" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I170" s="18"/>
-      <c r="J170" s="19"/>
-      <c r="K170" s="18"/>
+      <c r="I170" s="15"/>
+      <c r="J170" s="16"/>
+      <c r="K170" s="15"/>
     </row>
     <row r="171" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B171" s="17"/>
-      <c r="C171" s="21" t="s">
+      <c r="B171" s="14"/>
+      <c r="C171" s="11" t="s">
         <v>271</v>
       </c>
       <c r="D171" s="3" t="s">
@@ -5515,13 +5515,13 @@
       <c r="H171" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I171" s="18"/>
-      <c r="J171" s="19"/>
-      <c r="K171" s="18"/>
+      <c r="I171" s="15"/>
+      <c r="J171" s="16"/>
+      <c r="K171" s="15"/>
     </row>
     <row r="172" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B172" s="17"/>
-      <c r="C172" s="21" t="s">
+      <c r="B172" s="14"/>
+      <c r="C172" s="11" t="s">
         <v>272</v>
       </c>
       <c r="D172" s="3" t="s">
@@ -5539,13 +5539,13 @@
       <c r="H172" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I172" s="18"/>
-      <c r="J172" s="19"/>
-      <c r="K172" s="18"/>
+      <c r="I172" s="15"/>
+      <c r="J172" s="16"/>
+      <c r="K172" s="15"/>
     </row>
     <row r="173" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B173" s="17"/>
-      <c r="C173" s="21" t="s">
+      <c r="B173" s="14"/>
+      <c r="C173" s="11" t="s">
         <v>273</v>
       </c>
       <c r="D173" s="3" t="s">
@@ -5563,13 +5563,13 @@
       <c r="H173" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I173" s="18"/>
-      <c r="J173" s="19"/>
-      <c r="K173" s="18"/>
+      <c r="I173" s="15"/>
+      <c r="J173" s="16"/>
+      <c r="K173" s="15"/>
     </row>
     <row r="174" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B174" s="17"/>
-      <c r="C174" s="21" t="s">
+      <c r="B174" s="14"/>
+      <c r="C174" s="11" t="s">
         <v>274</v>
       </c>
       <c r="D174" s="3" t="s">
@@ -5587,13 +5587,13 @@
       <c r="H174" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I174" s="18"/>
-      <c r="J174" s="19"/>
-      <c r="K174" s="18"/>
+      <c r="I174" s="15"/>
+      <c r="J174" s="16"/>
+      <c r="K174" s="15"/>
     </row>
     <row r="175" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B175" s="17"/>
-      <c r="C175" s="21" t="s">
+      <c r="B175" s="14"/>
+      <c r="C175" s="11" t="s">
         <v>275</v>
       </c>
       <c r="D175" s="3" t="s">
@@ -5611,13 +5611,13 @@
       <c r="H175" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I175" s="18"/>
-      <c r="J175" s="19"/>
-      <c r="K175" s="18"/>
+      <c r="I175" s="15"/>
+      <c r="J175" s="16"/>
+      <c r="K175" s="15"/>
     </row>
     <row r="176" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B176" s="17"/>
-      <c r="C176" s="21" t="s">
+      <c r="B176" s="14"/>
+      <c r="C176" s="11" t="s">
         <v>276</v>
       </c>
       <c r="D176" s="3" t="s">
@@ -5635,13 +5635,13 @@
       <c r="H176" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I176" s="18"/>
-      <c r="J176" s="19"/>
-      <c r="K176" s="18"/>
+      <c r="I176" s="15"/>
+      <c r="J176" s="16"/>
+      <c r="K176" s="15"/>
     </row>
     <row r="177" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B177" s="17"/>
-      <c r="C177" s="21" t="s">
+      <c r="B177" s="14"/>
+      <c r="C177" s="11" t="s">
         <v>277</v>
       </c>
       <c r="D177" s="3" t="s">
@@ -5659,13 +5659,13 @@
       <c r="H177" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I177" s="18"/>
-      <c r="J177" s="19"/>
-      <c r="K177" s="18"/>
+      <c r="I177" s="15"/>
+      <c r="J177" s="16"/>
+      <c r="K177" s="15"/>
     </row>
     <row r="178" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B178" s="17"/>
-      <c r="C178" s="21" t="s">
+      <c r="B178" s="14"/>
+      <c r="C178" s="11" t="s">
         <v>278</v>
       </c>
       <c r="D178" s="3" t="s">
@@ -5683,13 +5683,13 @@
       <c r="H178" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I178" s="18"/>
-      <c r="J178" s="19"/>
-      <c r="K178" s="18"/>
+      <c r="I178" s="15"/>
+      <c r="J178" s="16"/>
+      <c r="K178" s="15"/>
     </row>
     <row r="179" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B179" s="17"/>
-      <c r="C179" s="21" t="s">
+      <c r="B179" s="14"/>
+      <c r="C179" s="11" t="s">
         <v>279</v>
       </c>
       <c r="D179" s="3" t="s">
@@ -5707,13 +5707,13 @@
       <c r="H179" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I179" s="18"/>
-      <c r="J179" s="19"/>
-      <c r="K179" s="18"/>
+      <c r="I179" s="15"/>
+      <c r="J179" s="16"/>
+      <c r="K179" s="15"/>
     </row>
     <row r="180" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B180" s="17"/>
-      <c r="C180" s="21" t="s">
+      <c r="B180" s="14"/>
+      <c r="C180" s="11" t="s">
         <v>280</v>
       </c>
       <c r="D180" s="3" t="s">
@@ -5731,29 +5731,29 @@
       <c r="H180" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I180" s="18"/>
-      <c r="J180" s="19"/>
-      <c r="K180" s="18"/>
+      <c r="I180" s="15"/>
+      <c r="J180" s="16"/>
+      <c r="K180" s="15"/>
     </row>
     <row r="181" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B181" s="17" t="s">
+      <c r="B181" s="14" t="s">
         <v>300</v>
       </c>
-      <c r="C181" s="20" t="s">
+      <c r="C181" s="12" t="s">
         <v>281</v>
       </c>
-      <c r="D181" s="15"/>
-      <c r="E181" s="15"/>
-      <c r="F181" s="15"/>
-      <c r="G181" s="15"/>
-      <c r="H181" s="15"/>
-      <c r="I181" s="15"/>
-      <c r="J181" s="15"/>
-      <c r="K181" s="15"/>
+      <c r="D181" s="13"/>
+      <c r="E181" s="13"/>
+      <c r="F181" s="13"/>
+      <c r="G181" s="13"/>
+      <c r="H181" s="13"/>
+      <c r="I181" s="13"/>
+      <c r="J181" s="13"/>
+      <c r="K181" s="13"/>
     </row>
     <row r="182" spans="2:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B182" s="17"/>
-      <c r="C182" s="21" t="s">
+      <c r="B182" s="14"/>
+      <c r="C182" s="11" t="s">
         <v>301</v>
       </c>
       <c r="D182" s="8" t="s">
@@ -5771,19 +5771,19 @@
       <c r="H182" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I182" s="18" t="s">
+      <c r="I182" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="J182" s="19" t="s">
+      <c r="J182" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K182" s="18" t="s">
+      <c r="K182" s="15" t="s">
         <v>290</v>
       </c>
     </row>
     <row r="183" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B183" s="17"/>
-      <c r="C183" s="21" t="s">
+      <c r="B183" s="14"/>
+      <c r="C183" s="11" t="s">
         <v>302</v>
       </c>
       <c r="D183" s="3" t="s">
@@ -5801,13 +5801,13 @@
       <c r="H183" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I183" s="18"/>
-      <c r="J183" s="19"/>
-      <c r="K183" s="18"/>
+      <c r="I183" s="15"/>
+      <c r="J183" s="16"/>
+      <c r="K183" s="15"/>
     </row>
     <row r="184" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B184" s="17"/>
-      <c r="C184" s="21" t="s">
+      <c r="B184" s="14"/>
+      <c r="C184" s="11" t="s">
         <v>303</v>
       </c>
       <c r="D184" s="3" t="s">
@@ -5825,13 +5825,13 @@
       <c r="H184" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I184" s="18"/>
-      <c r="J184" s="19"/>
-      <c r="K184" s="18"/>
+      <c r="I184" s="15"/>
+      <c r="J184" s="16"/>
+      <c r="K184" s="15"/>
     </row>
     <row r="185" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B185" s="17"/>
-      <c r="C185" s="21" t="s">
+      <c r="B185" s="14"/>
+      <c r="C185" s="11" t="s">
         <v>304</v>
       </c>
       <c r="D185" s="3" t="s">
@@ -5849,13 +5849,13 @@
       <c r="H185" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I185" s="18"/>
-      <c r="J185" s="19"/>
-      <c r="K185" s="18"/>
+      <c r="I185" s="15"/>
+      <c r="J185" s="16"/>
+      <c r="K185" s="15"/>
     </row>
     <row r="186" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B186" s="17"/>
-      <c r="C186" s="21" t="s">
+      <c r="B186" s="14"/>
+      <c r="C186" s="11" t="s">
         <v>305</v>
       </c>
       <c r="D186" s="3" t="s">
@@ -5873,13 +5873,13 @@
       <c r="H186" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I186" s="18"/>
-      <c r="J186" s="19"/>
-      <c r="K186" s="18"/>
+      <c r="I186" s="15"/>
+      <c r="J186" s="16"/>
+      <c r="K186" s="15"/>
     </row>
     <row r="187" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B187" s="17"/>
-      <c r="C187" s="21" t="s">
+      <c r="B187" s="14"/>
+      <c r="C187" s="11" t="s">
         <v>306</v>
       </c>
       <c r="D187" s="3" t="s">
@@ -5897,13 +5897,13 @@
       <c r="H187" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I187" s="18"/>
-      <c r="J187" s="19"/>
-      <c r="K187" s="18"/>
+      <c r="I187" s="15"/>
+      <c r="J187" s="16"/>
+      <c r="K187" s="15"/>
     </row>
     <row r="188" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B188" s="17"/>
-      <c r="C188" s="21" t="s">
+      <c r="B188" s="14"/>
+      <c r="C188" s="11" t="s">
         <v>307</v>
       </c>
       <c r="D188" s="3" t="s">
@@ -5921,13 +5921,13 @@
       <c r="H188" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I188" s="18"/>
-      <c r="J188" s="19"/>
-      <c r="K188" s="18"/>
+      <c r="I188" s="15"/>
+      <c r="J188" s="16"/>
+      <c r="K188" s="15"/>
     </row>
     <row r="189" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B189" s="17"/>
-      <c r="C189" s="21" t="s">
+      <c r="B189" s="14"/>
+      <c r="C189" s="11" t="s">
         <v>308</v>
       </c>
       <c r="D189" s="3" t="s">
@@ -5945,13 +5945,13 @@
       <c r="H189" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I189" s="18"/>
-      <c r="J189" s="19"/>
-      <c r="K189" s="18"/>
+      <c r="I189" s="15"/>
+      <c r="J189" s="16"/>
+      <c r="K189" s="15"/>
     </row>
     <row r="190" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B190" s="17"/>
-      <c r="C190" s="21" t="s">
+      <c r="B190" s="14"/>
+      <c r="C190" s="11" t="s">
         <v>309</v>
       </c>
       <c r="D190" s="3" t="s">
@@ -5969,13 +5969,13 @@
       <c r="H190" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I190" s="18"/>
-      <c r="J190" s="19"/>
-      <c r="K190" s="18"/>
+      <c r="I190" s="15"/>
+      <c r="J190" s="16"/>
+      <c r="K190" s="15"/>
     </row>
     <row r="191" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B191" s="17"/>
-      <c r="C191" s="21" t="s">
+      <c r="B191" s="14"/>
+      <c r="C191" s="11" t="s">
         <v>310</v>
       </c>
       <c r="D191" s="3" t="s">
@@ -5993,92 +5993,26 @@
       <c r="H191" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I191" s="18"/>
-      <c r="J191" s="19"/>
-      <c r="K191" s="18"/>
+      <c r="I191" s="15"/>
+      <c r="J191" s="16"/>
+      <c r="K191" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="109">
-    <mergeCell ref="C181:K181"/>
-    <mergeCell ref="B181:B191"/>
-    <mergeCell ref="I182:I191"/>
-    <mergeCell ref="J182:J191"/>
-    <mergeCell ref="K182:K191"/>
-    <mergeCell ref="C166:K166"/>
-    <mergeCell ref="B166:B180"/>
-    <mergeCell ref="I167:I180"/>
-    <mergeCell ref="J167:J180"/>
-    <mergeCell ref="K167:K180"/>
-    <mergeCell ref="B156:B165"/>
-    <mergeCell ref="C156:K156"/>
-    <mergeCell ref="I157:I165"/>
-    <mergeCell ref="J157:J165"/>
-    <mergeCell ref="K157:K165"/>
-    <mergeCell ref="C135:K135"/>
-    <mergeCell ref="I136:I155"/>
-    <mergeCell ref="J136:J155"/>
-    <mergeCell ref="K136:K155"/>
-    <mergeCell ref="B135:B155"/>
-    <mergeCell ref="B127:B134"/>
-    <mergeCell ref="C127:K127"/>
-    <mergeCell ref="I128:I134"/>
-    <mergeCell ref="J128:J134"/>
-    <mergeCell ref="K128:K134"/>
-    <mergeCell ref="B120:B126"/>
-    <mergeCell ref="C120:K120"/>
-    <mergeCell ref="I121:I126"/>
-    <mergeCell ref="J121:J126"/>
-    <mergeCell ref="K121:K126"/>
-    <mergeCell ref="B111:B119"/>
-    <mergeCell ref="C111:K111"/>
-    <mergeCell ref="I112:I119"/>
-    <mergeCell ref="J112:J119"/>
-    <mergeCell ref="K112:K119"/>
-    <mergeCell ref="B97:B110"/>
-    <mergeCell ref="C97:K97"/>
-    <mergeCell ref="I98:I110"/>
-    <mergeCell ref="J98:J110"/>
-    <mergeCell ref="K98:K110"/>
-    <mergeCell ref="B90:B96"/>
-    <mergeCell ref="C90:K90"/>
-    <mergeCell ref="I91:I96"/>
-    <mergeCell ref="J91:J96"/>
-    <mergeCell ref="K91:K96"/>
-    <mergeCell ref="B82:B89"/>
-    <mergeCell ref="C82:K82"/>
-    <mergeCell ref="I83:I89"/>
-    <mergeCell ref="J83:J89"/>
-    <mergeCell ref="K83:K89"/>
-    <mergeCell ref="C73:K73"/>
-    <mergeCell ref="B73:B81"/>
-    <mergeCell ref="I74:I81"/>
-    <mergeCell ref="J74:J81"/>
-    <mergeCell ref="K74:K81"/>
-    <mergeCell ref="B67:B72"/>
-    <mergeCell ref="C67:K67"/>
-    <mergeCell ref="I68:I72"/>
-    <mergeCell ref="J68:J72"/>
-    <mergeCell ref="K68:K72"/>
-    <mergeCell ref="B61:B66"/>
-    <mergeCell ref="C61:K61"/>
-    <mergeCell ref="I62:I66"/>
-    <mergeCell ref="J62:J66"/>
-    <mergeCell ref="K62:K66"/>
-    <mergeCell ref="B54:B60"/>
-    <mergeCell ref="C54:K54"/>
-    <mergeCell ref="I55:I60"/>
-    <mergeCell ref="J55:J60"/>
-    <mergeCell ref="K55:K60"/>
-    <mergeCell ref="B48:B53"/>
-    <mergeCell ref="C48:K48"/>
-    <mergeCell ref="I49:I53"/>
-    <mergeCell ref="J49:J53"/>
-    <mergeCell ref="K49:K53"/>
-    <mergeCell ref="B41:B47"/>
-    <mergeCell ref="C41:K41"/>
-    <mergeCell ref="I42:I47"/>
-    <mergeCell ref="J42:J47"/>
-    <mergeCell ref="K42:K47"/>
+    <mergeCell ref="B11:B18"/>
+    <mergeCell ref="I12:I18"/>
+    <mergeCell ref="J12:J18"/>
+    <mergeCell ref="K12:K18"/>
+    <mergeCell ref="C2:K2"/>
+    <mergeCell ref="C3:K3"/>
+    <mergeCell ref="C4:K4"/>
+    <mergeCell ref="C5:K5"/>
+    <mergeCell ref="C6:K6"/>
+    <mergeCell ref="C7:K7"/>
+    <mergeCell ref="C8:K8"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="C9:K9"/>
+    <mergeCell ref="C11:K11"/>
     <mergeCell ref="B34:B40"/>
     <mergeCell ref="C34:K34"/>
     <mergeCell ref="I35:I40"/>
@@ -6094,20 +6028,86 @@
     <mergeCell ref="I27:I33"/>
     <mergeCell ref="J27:J33"/>
     <mergeCell ref="K27:K33"/>
-    <mergeCell ref="B11:B18"/>
-    <mergeCell ref="I12:I18"/>
-    <mergeCell ref="J12:J18"/>
-    <mergeCell ref="K12:K18"/>
-    <mergeCell ref="C2:K2"/>
-    <mergeCell ref="C3:K3"/>
-    <mergeCell ref="C4:K4"/>
-    <mergeCell ref="C5:K5"/>
-    <mergeCell ref="C6:K6"/>
-    <mergeCell ref="C7:K7"/>
-    <mergeCell ref="C8:K8"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="C9:K9"/>
-    <mergeCell ref="C11:K11"/>
+    <mergeCell ref="B48:B53"/>
+    <mergeCell ref="C48:K48"/>
+    <mergeCell ref="I49:I53"/>
+    <mergeCell ref="J49:J53"/>
+    <mergeCell ref="K49:K53"/>
+    <mergeCell ref="B41:B47"/>
+    <mergeCell ref="C41:K41"/>
+    <mergeCell ref="I42:I47"/>
+    <mergeCell ref="J42:J47"/>
+    <mergeCell ref="K42:K47"/>
+    <mergeCell ref="B61:B66"/>
+    <mergeCell ref="C61:K61"/>
+    <mergeCell ref="I62:I66"/>
+    <mergeCell ref="J62:J66"/>
+    <mergeCell ref="K62:K66"/>
+    <mergeCell ref="B54:B60"/>
+    <mergeCell ref="C54:K54"/>
+    <mergeCell ref="I55:I60"/>
+    <mergeCell ref="J55:J60"/>
+    <mergeCell ref="K55:K60"/>
+    <mergeCell ref="C73:K73"/>
+    <mergeCell ref="B73:B81"/>
+    <mergeCell ref="I74:I81"/>
+    <mergeCell ref="J74:J81"/>
+    <mergeCell ref="K74:K81"/>
+    <mergeCell ref="B67:B72"/>
+    <mergeCell ref="C67:K67"/>
+    <mergeCell ref="I68:I72"/>
+    <mergeCell ref="J68:J72"/>
+    <mergeCell ref="K68:K72"/>
+    <mergeCell ref="B90:B96"/>
+    <mergeCell ref="C90:K90"/>
+    <mergeCell ref="I91:I96"/>
+    <mergeCell ref="J91:J96"/>
+    <mergeCell ref="K91:K96"/>
+    <mergeCell ref="B82:B89"/>
+    <mergeCell ref="C82:K82"/>
+    <mergeCell ref="I83:I89"/>
+    <mergeCell ref="J83:J89"/>
+    <mergeCell ref="K83:K89"/>
+    <mergeCell ref="B111:B119"/>
+    <mergeCell ref="C111:K111"/>
+    <mergeCell ref="I112:I119"/>
+    <mergeCell ref="J112:J119"/>
+    <mergeCell ref="K112:K119"/>
+    <mergeCell ref="B97:B110"/>
+    <mergeCell ref="C97:K97"/>
+    <mergeCell ref="I98:I110"/>
+    <mergeCell ref="J98:J110"/>
+    <mergeCell ref="K98:K110"/>
+    <mergeCell ref="B127:B134"/>
+    <mergeCell ref="C127:K127"/>
+    <mergeCell ref="I128:I134"/>
+    <mergeCell ref="J128:J134"/>
+    <mergeCell ref="K128:K134"/>
+    <mergeCell ref="B120:B126"/>
+    <mergeCell ref="C120:K120"/>
+    <mergeCell ref="I121:I126"/>
+    <mergeCell ref="J121:J126"/>
+    <mergeCell ref="K121:K126"/>
+    <mergeCell ref="B156:B165"/>
+    <mergeCell ref="C156:K156"/>
+    <mergeCell ref="I157:I165"/>
+    <mergeCell ref="J157:J165"/>
+    <mergeCell ref="K157:K165"/>
+    <mergeCell ref="C135:K135"/>
+    <mergeCell ref="I136:I155"/>
+    <mergeCell ref="J136:J155"/>
+    <mergeCell ref="K136:K155"/>
+    <mergeCell ref="B135:B155"/>
+    <mergeCell ref="C181:K181"/>
+    <mergeCell ref="B181:B191"/>
+    <mergeCell ref="I182:I191"/>
+    <mergeCell ref="J182:J191"/>
+    <mergeCell ref="K182:K191"/>
+    <mergeCell ref="C166:K166"/>
+    <mergeCell ref="B166:B180"/>
+    <mergeCell ref="I167:I180"/>
+    <mergeCell ref="J167:J180"/>
+    <mergeCell ref="K167:K180"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>